<commit_message>
Split tools into 6 separate files (one tool per file)
app/tools/
  check_delay.py         - check_delay_threshold
  check_baggage.py       - check_baggage_threshold
  refund_calculator.py   - calculate_refund
  timeline_calculator.py - calculate_refund_timeline
  letter.py              - generate_decision_letter
  search.py              - search_regulations + get_all_tools

Co-authored-by: mattkaplanai <mattkaplanai@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/decision_log.xlsx
+++ b/decision_log.xlsx
@@ -559,12 +559,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-02-27 21:53:05</t>
+          <t>2026-02-28 05:21:58</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Flight Cancellation</t>
+          <t>Schedule Change / Significant Delay</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -584,7 +584,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>My JetBlue flight B6 401 from Boston to Fort Lauderdale on March 15 was cancelled. The airline offered me a voucher but I said no.</t>
+          <t>My flight was delayed a lot and I missed my meeting. The airline didn't help at all. I think I deserve my money back. It was sometime last month.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -594,45 +594,48 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Step 1 — Searched DOT regulations regarding flight cancellations.
-Step 2 — Determined that the flight was cancelled and no alternative transportation was accepted.
-Step 3 — Calculated the refund timeline for credit card payments.</t>
+          <t>Step 1 — Confirmed that the flight delay was significant, exceeding the 3-hour threshold.
+Step 2 — Verified that the passenger did not accept any alternative offered by the airline.
+Step 3 — Determined that the passenger is entitled to a refund as per DOT regulations.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Passenger did not accept alternative transportation, but the decision should reflect that a refund is not warranted if alternatives were offered.</t>
+          <t>Insufficient evidence of significant delay as per the threshold requirements.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>14 CFR part 260
-§ 260.6</t>
+          <t>14 CFR Part 260
+USDOT Aviation Refunds
+14 CFR Part 259</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>full fare</t>
+          <t>ticket refund</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>credit_card</t>
+          <t>Credit Card</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Refund must be issued within 7 business days after the refund becomes due.</t>
+          <t>within 7 business days</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>Wait for the refund to be processed within the specified timeline.</t>
+          <t>Wait for the airline to process the refund within the specified timeline.
+Contact the airline if the refund is not received within 7 business days.
+Keep a record of all communications with the airline regarding the refund.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync: config, RAG, refund agent, docs, scripts, bilgiler and .gitignore updates
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/decision_log.xlsx
+++ b/decision_log.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Refund Decisions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Refund Decisions'!$A$1:$P$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Refund Decisions'!$A$1:$Q$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -36,7 +36,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -51,8 +51,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
         <bgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -83,6 +95,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -450,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -459,16 +477,17 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="50" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
-    <col width="25" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
     <col width="25" customWidth="1" min="15" max="15"/>
-    <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,50 +523,55 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Accepted Alternative</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Analysis Steps</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Reasons</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Applicable Regulations</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Refund Type</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Refund Payment</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Refund Timeline</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Passenger Action Items</t>
         </is>
@@ -559,7 +583,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-02-28 05:21:58</t>
+          <t>2026-03-04 00:21:02</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -584,63 +608,1589 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>My flight was delayed a lot and I missed my meeting. The airline didn't help at all. I think I deserve my money back. It was sometime last month.</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>I booked a non-refundable round-trip ticket on Delta Air Lines from New York (JFK) to Los Angeles (LAX) for $450, paid by credit card. My outbound flight was DL 287 on March 15, 2025, scheduled to dep</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Verified the flight delay duration of 4.75 hours exceeds the DOT threshold of 3 hours for domestic flights.
+Step 2 — Confirmed the passenger did not accept any alternative transportation and did not use the outbound segment.
+Step 3 — Determined the passenger is eligible for a full refund of the outbound segment despite the non-refundable ticket.
+Step 4 — Established refund timeline of 7 business days for credit card payments as per DOT regulations.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>The flight delay of 4.75 hours exceeds the DOT significant delay threshold of 3 hours for domestic flights.
+The passenger did not accept any alternative transportation and did not use the outbound segment, making them eligible for a full refund of $450.</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>The U.S. Department of Transportation (DOT) requires airlines to provide refunds for significant delays.
+Mechanical issues causing significant delays entitle passengers to refunds even on non-refundable tickets.
+Refunds must be processed within 7 business days for credit card payments.</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Full refund of outbound segment</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Within 7 business days from 2025-03-15</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>Expect the refund of $450.00 to be processed to your credit card within 7 business days from March 15, 2025.
+If you do not receive the refund within this timeframe, contact Delta Air Lines customer service for follow-up.
+If the refund is not resolved, consider filing a complaint with the U.S. Department of Transportation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04 00:34:43</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Baggage Lost or Delayed</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Domestic (within US)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I flew United from Chicago to Denver. My checked bag did not arrive with the flight. I had to wait 8 hours at the airport before they delivered it. The bag had my work laptop and medication inside. I </t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>DENIED</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Step 1 — Confirmed that the flight delay was significant, exceeding the 3-hour threshold.
-Step 2 — Verified that the passenger did not accept any alternative offered by the airline.
-Step 3 — Determined that the passenger is entitled to a refund as per DOT regulations.</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Insufficient evidence of significant delay as per the threshold requirements.</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>14 CFR Part 260
-USDOT Aviation Refunds
-14 CFR Part 259</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>ticket refund</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>Credit Card</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>within 7 business days</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>Wait for the airline to process the refund within the specified timeline.
-Contact the airline if the refund is not received within 7 business days.
-Keep a record of all communications with the airline regarding the refund.</t>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Checked the baggage delay duration against the DOT threshold for significant delay on domestic flights.
+Step 2 — Determined that the baggage delay was 8 hours, which is less than the 12-hour threshold.
+Step 3 — Concluded that the passenger is not entitled to a refund or compensation for the baggage delay.
+Step 4 — Verified that the baggage fee refund is not warranted under DOT rules for this delay duration.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Baggage delay of 8 hours does not meet DOT threshold for significant delay on domestic flights.
+Passenger is not entitled to refund or compensation for baggage delay under DOT regulations.</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>DOT regulations on baggage delay compensation and refund for baggage fee</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>No refund or compensation will be issued for the baggage delay.
+If you have incurred reasonable expenses due to the baggage delay, you may submit receipts to United for consideration under their policies.
+If you disagree with this decision, you may file a complaint with the U.S. Department of Transportation at https://airconsumer.dot.gov.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04 00:48:39</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Schedule Change / Significant Delay</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Domestic (within US)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>My American Airlines flight from Dallas to Miami on February 20, 2025 was supposed to leave at 6:00 PM but we did not take off until 10:30 PM because of a maintenance delay. I paid $380 for the ticket</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>DENIED</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Verified the flight delay duration of 4.5 hours exceeds the 3-hour threshold for domestic flights.
+Step 2 — Confirmed the passenger did not accept any alternative voucher or rebooking.
+Step 3 — Calculated the full refund amount of $380 based on the ticket price and unused value.
+Step 4 — Determined refund deadline as 7 business days after flight date, by 2025-03-03.
+Step 5 — Applied DOT regulations supporting refund eligibility for significant delays caused by maintenance.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Passenger traveled on the delayed flight and did not accept any alternative voucher or rebooking, so refund is generally not warranted.
+DOT regulations do not require refund for passengers who complete travel on delayed flights unless there is a downgrade or other service failure.
+The ticket was non-refundable and the passenger used the service, so refund is not justified despite the delay.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Domestic Flight Delay Refunds
+Maintenance Delays
+Credit Card Payment Refunds</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Full refund</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Refund must be issued within 7 business days after 2025-02-20, by 2025-03-03</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>Send the formal refund request letter to American Airlines customer relations.
+Keep a copy of all correspondence and receipts related to this refund request.
+If the refund is not received by 2025-03-03, file a complaint with the U.S. Department of Transportation at https://airconsumer.dot.gov.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04 01:11:51</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Schedule Change / Significant Delay</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Domestic (within US)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>I bought a non-refundable ticket on United from Houston to Newark for $320, paid by credit card. Flight UA 156 on January 10, 2025 was supposed to leave at 2:00 PM but we did not take off until 6:30 P</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Confirm the flight delay duration meets the DOT threshold for significant delay (3+ hours for domestic flights).
+Step 2 — Verify the passenger did not accept any alternative transportation or vouchers.
+Step 3 — Confirm the passenger did not travel on the delayed flight.
+Step 4 — Determine the refund amount equals the full ticket price paid by credit card.
+Step 5 — Set refund deadline as 7 business days from the flight date.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>The flight delay of 4.5 hours qualifies as significant under DOT rules for domestic flights.
+The passenger did not accept rebooking or vouchers and did not travel.
+Passenger is entitled to a full refund of the ticket price paid by credit card.
+Refund must be issued within 7 business days of the refund becoming due.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>14 CFR Part 259 — significant delay refund requirement (domestic 4+ hours)</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Full refund</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>Within 7 business days from January 10, 2025</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>Send the formal refund request letter to United Airlines Customer Relations.
+Keep a copy of the letter and any correspondence with the airline.
+If the refund is not received within 7 business days, file a complaint with the U.S. Department of Transportation at https://airconsumer.dot.gov.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04 01:21:24</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Baggage Lost or Delayed</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Domestic (within US)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I flew Southwest from Phoenix to Denver. My checked bag did not show up at the carousel. I waited 14 hours at the airport before they delivered it. I paid $30 for the bag. I want a refund for the bag </t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Confirm baggage delay duration: 14 hours.
+Step 2 — Compare delay to threshold for domestic flights: 14 hours &gt; 12 hours threshold.
+Step 3 — Determine refund eligibility: Delay qualifies as significant, passenger entitled to baggage fee refund.
+Step 4 — Calculate refund amount: Full baggage fee of $30.
+Step 5 — Confirm payment method and refund timeline: Credit card payment, refund within 7 business days.
+Step 6 — Final recommendation: Approve refund of $30.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>The baggage delay of 14 hours exceeds the 12-hour threshold for domestic flights, qualifying as a significant delay.
+The passenger paid a $30 baggage fee and did not accept any alternative compensation.
+Under 14 CFR Part 254, airlines must compensate passengers for reasonable expenses due to baggage delays, including refunding baggage fees for significant delays.
+Refund should be processed within 7 business days as per credit card refund rules.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>14 CFR Part 254 — Airlines must compensate for reasonable expenses due to baggage delays, including refunding baggage fees for significant delays.</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Baggage fee refund</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>Refund must be issued within 7 business days</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>Send the formal refund request letter to Southwest Customer Relations.
+Keep a copy of the letter and any correspondence for your records.
+Monitor your credit card statement for the refund within 7 business days.
+If the refund is not received within the timeframe, consider filing a complaint with the U.S. Department of Transportation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04 20:40:24</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Flight Cancellation</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Domestic (within US)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>British Airways cancelled my flight from London Heathrow to New York JFK on April 5, 2025. I had paid £680 for the round-trip, by credit card. They offered me a rebook two days later but I declined. I</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Verified that the flight was canceled by the airline.
+Step 2 — Confirmed the passenger did not accept the alternative rebooking offered.
+Step 3 — Confirmed the passenger did not travel on the flight.
+Step 4 — Applied DOT rules requiring full refund for cancellations without accepted alternatives.
+Step 5 — Determined refund amount as full ticket price $680.
+Step 6 — Set refund deadline as 7 business days after cancellation date (April 15, 2025).</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Flight was canceled by the airline
+Passenger did not accept the offered rebooking
+Passenger did not travel
+DOT rules require full refund for cancellations without accepted alternatives</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>14 CFR 374.3 — Refunds for Canceled Flights
+14 CFR 259.5 — Prompt Refunds for Canceled Flights</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Full refund</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>Refund must be issued within 7 business days of cancellation date (by April 15, 2025)</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>Send the formal refund request letter to British Airways customer relations.
+Keep a copy of all correspondence with the airline.
+If refund is not received by April 15, 2025, file a complaint with the U.S. Department of Transportation at https://airconsumer.dot.gov.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04 20:53:28</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Flight Cancellation</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Domestic (within US)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>I had a non-refundable American Airlines ticket from Miami to Boston, $290 paid by credit card. Flight AA 842 on May 12, 2025 was delayed over 5 hours due to mechanical issues. I did not accept rebook</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>DENIED</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Verified the flight delay duration of 5 hours exceeds the 3-hour threshold for significant delays on domestic flights.
+Step 2 — Confirmed the passenger did not accept any alternative rebooking or voucher offers.
+Step 3 — Determined the passenger is entitled to a full refund of the ticket price under DOT regulations.
+Step 4 — Established refund amount as $290.00, to be refunded to the original credit card payment method.
+Step 5 — Set refund timeline to within 7 business days from the flight date, per DOT rules.</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Passenger traveled on the delayed flight and did not accept rebooking or voucher, so no refund is due under DOT regulations for delay alone.
+DOT refund rules for significant delays apply primarily when the passenger does not travel or accepts a refund instead of traveling.
+No downgrade or other compensable issue was indicated to justify a refund despite traveling.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>14 CFR Part 259 — outlines refund requirements for significant delays (domestic flights).</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Full refund</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>Refund due within 7 business days from May 12, 2025</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>Send the formal refund request letter to American Airlines Customer Relations.
+Keep a copy of the letter and any correspondence for your records.
+Monitor your credit card statement for the refund within 7 business days.
+If the refund is not received within the timeframe, file a complaint with the U.S. Department of Transportation at https://airconsumer.dot.gov.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04 21:00:56</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Flight Cancellation</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Domestic (within US)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>British Airways delayed my flight from New York to London by 5 hours. I did not accept vouchers. I paid $900 by credit card and want a refund under DOT rules.</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>DENIED</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Verified the flight delay duration is 5 hours.
+Step 2 — Compared delay duration against DOT threshold of 6 hours for international flights.
+Step 3 — Determined the delay does not meet the significant delay threshold for refund entitlement.
+Step 4 — Confirmed passenger did not accept alternative arrangements or vouchers.
+Step 5 — Concluded no refund is due based on DOT regulations for delay under 6 hours.</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>The delay of 5.0 hours does NOT meet the 6.0-hour threshold for international flights.
+The delay is NOT considered significant — no refund entitlement based on delay alone.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>14 CFR Part 259 — Airline obligations to passengers in the event of delays and cancellations</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>Review the DOT regulations on airline delay refunds for international flights.
+Contact British Airways customer service for any further clarifications.
+If you believe your case has special circumstances, consider filing a complaint with the U.S. Department of Transportation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04 21:10:50</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Downgrade to Lower Class</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Domestic (within US)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>I was downgraded from business to economy on my international flight. I paid $1,200 for business. I want a refund for the difference.</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Confirmed the passenger was downgraded from business to economy on an international flight.
+Step 2 — Verified the passenger paid $1200 for business class and traveled in economy.
+Step 3 — Calculated refund amount as the fare difference, $1200.
+Step 4 — Confirmed refund timeline for credit card payments is within 7 business days.
+Step 5 — Recommended approval based on regulations and refund calculation.</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Passenger is entitled to a refund for the fare difference between business and economy class, not the full business class fare.
+Without the economy class fare, the refund amount cannot be accurately determined.
+The decision should be partial approval pending correct fare difference calculation and proper regulation citation.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Please refer to the DOT's official resources or contact them for specific guidance on downgrades and refunds for international flights</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Fare difference refund</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>Within 7 business days</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>Submit the formal refund request letter to the airline's customer relations department.
+Keep a copy of all correspondence with the airline.
+Monitor your credit card statement for the refund within 7 business days.
+If the refund is not received within the timeline, consider filing a complaint with the U.S. Department of Transportation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04 21:11:59</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Flight Cancellation</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Domestic (within US)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>The airline cancelled my international flight to London. They offered a flight 2 days later but I could not accept. I paid $650 and did not travel. I want a full refund.</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Confirm flight cancellation by airline.
+Step 2 — Verify passenger did not accept offered alternative flight.
+Step 3 — Confirm passenger did not travel on the original or alternative flight.
+Step 4 — Calculate refund amount as full ticket price of $650.00.
+Step 5 — Determine refund timeline as 7 business days due to credit card payment.
+Step 6 — Apply DOT regulation 14 CFR Part 259 requiring full refund for canceled flights with no accepted alternative.</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>The airline canceled the international flight.
+The passenger declined the offered alternative flight.
+The passenger did not travel.
+DOT regulations require a full refund in such cases.
+The refund amount matches the full ticket price paid.
+Refund must be issued within 7 business days for credit card payments.</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>14 CFR Part 259 — Airlines must provide a full refund for canceled flights if no alternative is accepted by the passenger.</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>Full refund</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>Within 7 business days</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>Submit the formal refund request letter to the airline's customer service department.
+Keep a copy of all correspondence with the airline.
+Monitor your credit card statement for the refund within 7 business days.
+If the refund is not received within the required timeframe, file a complaint with the U.S. Department of Transportation at https://airconsumer.dot.gov.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04 21:21:06</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>24-Hour Cancellation (within 24h of booking)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Domestic (within US)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>I booked a domestic flight and cancelled within 6 hours of booking. I want my money back under the 24-hour rule.</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Confirmed cancellation was within 24 hours of booking.
+Step 2 — Verified flight was domestic and passenger did not travel.
+Step 3 — Confirmed no alternative was accepted by the passenger.
+Step 4 — Calculated full refund amount including ticket price and taxes/fees.
+Step 5 — Determined refund timeline based on payment method (credit card).</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Passenger canceled within the 24-hour cancellation window for a domestic flight
+Passenger did not travel
+Passenger did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>14 CFR Part 259 — Requirements for airlines regarding consumer protection including the 24-hour cancellation policy</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>Full refund</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>Refund must be issued within 7 business days</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>Send the formal refund request letter to the airline's customer relations department.
+Keep a copy of the letter and any correspondence with the airline.
+Monitor your credit card statement for the refund within 7 business days.
+If refund is not received within the timeframe, consider filing a complaint with the U.S. Department of Transportation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04 21:22:54</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Flight Cancellation</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Domestic (within US)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>My domestic flight from Chicago to Dallas was delayed 4 hours. I did not accept rebooking. I paid $280 by credit card and want a refund.</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>DENIED</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Confirm the flight delay duration meets the threshold for a significant delay (3+ hours for domestic flights).
+Step 2 — Verify the passenger did not accept any alternative rebooking offered by the airline.
+Step 3 — Confirm the passenger did not travel any segments of the flight.
+Step 4 — Determine the refund amount equals the full ticket price since no segments were used.
+Step 5 — Confirm the refund must be processed within 7 business days as payment was made by credit card.</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Passenger traveled on the flight despite the delay, so refund is not warranted under DOT rules for delay refund.
+Analysis incorrectly concluded no segments were traveled, leading to an erroneous refund approval.
+No downgrade or other compensable issue present to justify refund despite travel.
+Incomplete decision letter details reduce clarity and formal validity.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>14 CFR 259.4 — significant delay refund requirement (domestic 3+ hours)</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Full refund</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>Refund must be issued within 7 business days</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>Submit the formal refund request letter to the airline's customer service department.
+Keep a copy of all correspondence with the airline regarding this refund.
+If the refund is not received within 7 business days, consider filing a complaint with the U.S. Department of Transportation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04 21:25:55</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Baggage Lost or Delayed</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Domestic (within US)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>My checked bag was delayed 14 hours on a domestic flight. I had to buy essentials for $75. I want reimbursement for the bag fee and my expenses.</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Verified baggage delay duration: 14 hours.
+Step 2 — Compared delay to threshold for domestic flights: 12 hours.
+Step 3 — Determined delay exceeds threshold, qualifying as significant delay.
+Step 4 — Confirmed passenger is entitled to reimbursement for baggage fee and reasonable expenses.
+Step 5 — Noted no ticket refund applicable due to lack of ticket price or fees provided.
+Step 6 — Recommended refund approval with refund to be issued within 7 business days.</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>The baggage delay of 14 hours exceeds the 12-hour threshold for domestic flights, qualifying as a significant delay.
+Passenger is entitled to reimbursement for the baggage fee and reasonable expenses incurred due to the delay.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Department of Transportation regulations on baggage delay compensation
+Airline policies on baggage fee refund for delays over 12 hours</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Baggage fee and reimbursement for essentials</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>Refund must be issued within 7 business days</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>Send the formal refund request letter to the airline's customer relations department.
+Keep copies of all receipts related to expenses incurred due to baggage delay.
+Monitor for refund confirmation within 7 business days.
+If refund is not received within the timeframe, consider filing a complaint with the U.S. Department of Transportation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-05 02:02:36</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Flight Cancellation</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Domestic (within US)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>My checked bag was delayed 20 hours on an international flight from Frankfurt to New York. I had to buy clothes and toiletries. I paid 120 EUR for essentials and 65 EUR for the bag fee. I want reimbur</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Verified baggage delay duration of 20 hours exceeds the 15-hour threshold for significant delay.
+Step 2 — Converted essential expenses of 120 EUR to $139.79 USD and baggage fee of 65 EUR to $75.72 USD.
+Step 3 — Confirmed passenger is entitled to reimbursement of baggage fee and supported claim for essentials under Montreal Convention.
+Step 4 — Confirmed refund timeline for credit card payments is 7 business days.</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Passenger is entitled to reimbursement of the baggage fee paid due to baggage delay exceeding 15 hours on an international flight under Montreal Convention.
+Reimbursement of essential expenses requires further proof and is subject to liability limits; cannot be approved without additional documentation and airline acceptance.
+Refund amount should be limited to baggage fee refund unless further claims are substantiated.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Montreal Convention (1999) — Article 19 — carrier liability for delay in carriage of passengers, baggage or cargo.
+Montreal Convention (1999) — Article 22 — liability limits for baggage (amounts expressed in SDRs).</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>Baggage fee refund</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>Refund must be issued within 7 business days after the refund becomes due.</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>Submit the formal refund request letter to the airline's customer relations department.
+Keep receipts and documentation of essential expenses for potential further claims.
+Monitor for refund confirmation within 7 business days.
+If refund is not received within the timeframe, file a complaint with the U.S. Department of Transportation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-05 02:13:32</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Flight Cancellation</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>The airline cancelled my domestic flight 2 days before departure. I did not accept rebooking or voucher. I paid $340 for the ticket and want a full refund.</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Confirmed flight was canceled by the airline.
+Step 2 — Verified passenger did not accept alternative transportation or voucher.
+Step 3 — Confirmed passenger did not travel on the flight.
+Step 4 — Checked payment method was credit card.
+Step 5 — Applied DOT regulations requiring full refund to original form of payment for canceled flights when alternatives are declined.
+Step 6 — Determined refund amount as full ticket price $340.00 USD.
+Step 7 — Recommended refund approval with processing within 7 business days.</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>The airline canceled the domestic flight and the passenger did not accept any alternative transportation or voucher.
+Under DOT rules (14 CFR Part 259 and 259.5), the passenger is entitled to a full refund of the unused ticket price despite the ticket being non-refundable.
+The refund must be processed promptly to the original form of payment (credit card) within 7 business days.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>14 CFR Part 259 — Enhancing Airline Passenger Protections
+14 CFR 259.5 — Refunds (carrier cancellation — refund required)
+DOT Final Rule — Enhancing Airline Passenger Protections (Federal Register) — implementing 14 CFR Part 259
+DOT guidance on refund timeliness (credit-card refunds — prompt processing, commonly 7 business days)</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Full refund of unused ticket fare</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>Refund must be processed within 7 business days to the original form of payment</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>Submit the formal refund request letter to the airline's customer relations department.
+Keep a copy of all correspondence with the airline regarding this refund.
+If the refund is not received within 7 business days, file a complaint with the U.S. Department of Transportation at https://airconsumer.dot.gov.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-05 02:15:16</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Schedule Change / Significant Delay</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>My international flight was delayed 7 hours at departure. I did not accept rebooking. I paid 450 EUR for the ticket. I want a full refund in USD.</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>DENIED</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Confirmed the flight delay duration of 7 hours exceeds the 6-hour threshold for significant delay on international flights.
+Step 2 — Verified the passenger did not accept rebooking, making them eligible for a refund.
+Step 3 — Converted the ticket price from 450 EUR to $524.21 USD using the provided exchange rate.
+Step 4 — Confirmed refund must be issued within 7 business days as per credit card payment rules.
+Step 5 — Recommended full refund approval based on DOT rules and case facts.</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>DOT regulations require refunds to be issued in the original form of payment and currency; converting to USD is incorrect and may cause issues.
+The refund request letter is incomplete and contains inaccurate statements about currency conversion.
+The refund amount should be refunded in EUR as per DOT rules, so the current approval with USD refund is not compliant.</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>The DOT’s refund/consumer-protection rules require carriers to offer refunds when a flight is significantly delayed or cancelled and the passenger chooses not to travel — this applies even for non-refundable fares
+A 7-hour departure delay on an international flight meets the significant delay threshold that triggers the refund requirement if the passenger declines transport
+Refunds must be provided in the original form of payment (credit card) rather than as a travel credit
+DOT rules do not require the carrier to convert the refund amount into a different currency; the customary practice is to refund in the original currency/payment form</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>Full refund</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>Refund must be issued within 7 business days</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>Send the formal refund request letter to the airline's customer relations department.
+Keep a copy of the letter and any correspondence with the airline.
+Monitor your credit card statement for the refund within 7 business days.
+If the refund is not received within the required timeframe, file a complaint with the U.S. Department of Transportation at https://airconsumer.dot.gov.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-05 02:24:30</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Baggage Lost or Delayed</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Non-refundable</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>No — I did not accept any alternative</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>My bag was delayed 22 hours on an international flight (about 9 hours). I paid 95 EUR for essentials and 55 EUR bag fee. I want reimbursement in USD.</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>DENIED</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Step 1 — Confirm baggage delay exceeds threshold: 22 hours delay &gt; 15 hours threshold for this flight.
+Step 2 — Convert expenses from EUR to USD: essentials EUR 95 = $110.67 USD, baggage fee EUR 55 = $64.07 USD.
+Step 3 — Determine refund eligibility: ancillary baggage fee refundable, essentials expense reimbursable under Montreal Convention.
+Step 4 — Confirm refund method and timeline: refund to original credit card within 7 business days.</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Passenger traveled on the flight and did not accept alternative, so no refund is due for baggage delay under policy.
+No downgrade or class difference to justify refund.
+Threshold correctly applied but passenger action disqualifies refund.</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Montreal Convention (1999), Article 19 — carrier liability for damage occasioned by delay
+Montreal Convention (1999), Article 22 — limits of liability for baggage
+14 CFR Part 259 (DOT) — consumer protections on refunds and prompt refund mechanics
+14 CFR 259.5 (or DOT rule within Part 259) — prompt refunds to the original form of payment when refund is due
+49 U.S.C. § 41712 — prohibition on unfair or deceptive practices</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>Baggage fee refund and essentials reimbursement</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Credit Card</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>Refund must be issued within 7 business days after refund due date</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>Submit the formal refund request letter to the airline's customer relations department.
+Keep copies of all receipts and correspondence related to the baggage delay and expenses.
+Monitor your credit card statement for the refund within 7 business days.
+If refund is not received within the timeframe, file a complaint with the U.S. Department of Transportation.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P2"/>
+  <autoFilter ref="A1:Q18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>